<commit_message>
Updating made to main run for in report
</commit_message>
<xml_diff>
--- a/study_case_model/scenario_variables/other_experiment_data/demand_scenarios155.xlsx
+++ b/study_case_model/scenario_variables/other_experiment_data/demand_scenarios155.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>19789.65151683206</v>
+        <v>28725.35614758425</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>21930.38171415172</v>
+        <v>23963.01774121611</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10534.66850774528</v>
+        <v>14928.8320178776</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>20914.12923220233</v>
+        <v>29138.17913844815</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5228.532308050583</v>
+        <v>7284.544784612039</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>37663.70101426699</v>
+        <v>46487.69937914996</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>16703.86500246677</v>
+        <v>11621.98641144057</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>25001.55298688648</v>
+        <v>36844.09611630544</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>24930.24759146039</v>
+        <v>30755.76046864681</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>11270.39481307656</v>
+        <v>10739.47105274393</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>20931.14410315387</v>
+        <v>23255.36026151579</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5232.786025788469</v>
+        <v>5813.840065378947</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>62376.47397001452</v>
+        <v>43048.73460781306</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>9248.261691084124</v>
+        <v>10753.51342411154</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>20064.12633193557</v>
+        <v>26814.71703674526</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>22722.05478417502</v>
+        <v>10650.39816506652</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>7452.984036975444</v>
+        <v>6031.558128076127</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>15084.45284167102</v>
+        <v>16626.27482455417</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>3771.113210417754</v>
+        <v>4156.568706138542</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>42856.68689683011</v>
+        <v>34807.53319498364</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>15778.95942767273</v>
+        <v>13678.42749723228</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>26969.20996751443</v>
+        <v>18189.81943359092</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>26451.92433525658</v>
+        <v>14407.72223998532</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>15690.8673581299</v>
+        <v>17996.18288345583</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>19175.76926960362</v>
+        <v>18645.34219708079</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>4793.942317400905</v>
+        <v>4661.335549270197</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>55856.97274893335</v>
+        <v>51012.92307031886</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>12112.91842650314</v>
+        <v>7157.194301699537</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>26990.21762049721</v>
+        <v>20917.12956606113</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>20629.31006791313</v>
+        <v>25831.91942282399</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>3354.435656463391</v>
+        <v>8183.774084666365</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>19194.32502688218</v>
+        <v>22254.18811007404</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>4798.581256720544</v>
+        <v>5563.547027518509</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>71341.2220414991</v>
+        <v>40990.41965121793</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>15973.30775840597</v>
+        <v>11406.14843827521</v>
       </c>
     </row>
     <row r="90">

</xml_diff>